<commit_message>
auto: 2026-03-17 09:45 (1 files)
</commit_message>
<xml_diff>
--- a/PantherBet_Bonuses.xlsx
+++ b/PantherBet_Bonuses.xlsx
@@ -6345,7 +6345,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>1 FS</t>
+          <t>100 FS</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr">
@@ -6381,7 +6381,7 @@
       </c>
       <c r="N101" s="5" t="inlineStr">
         <is>
-          <t>bonus_value: 100 FS vs 1 FS; game: endorphina2_BookOfSanta vs JokersJewels; available: 2025-11-28 - 2025-11-29 vs 2025-11-29 - 2025-11-30; identifier: blackfriday_day_5_fs_bonus_3_fs_title vs blackfriday_day_6_fs_bonus_3_fs_title</t>
+          <t>bonus_value: 100 FS vs 100 FS; game: endorphina2_BookOfSanta vs JokersJewels; available: 2025-11-28 - 2025-11-29 vs 2025-11-29 - 2025-11-30; identifier: blackfriday_day_5_fs_bonus_3_fs_title vs blackfriday_day_6_fs_bonus_3_fs_title</t>
         </is>
       </c>
     </row>

</xml_diff>